<commit_message>
fix(docbuilder/demo): regenerate base files — add Heading 1/Table Grid styles to docx, add Summary branding rows to xlsx
Closes the base-file asset gap flagged across t1, t2, t3:
- proposal_v1.docx: rebuilt with standard named styles so table_style "Table Grid"
  and Heading 1 apply (no more defensive fallback warnings on render)
- proposal_v1.xlsx: Summary sheet now has logo (row 1) + navy separator (row 2) +
  header fill (row 3) branding matching Line Items

Full suite 141 passed; branded docx render is now warning-free.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docbuilder/data/templates/demo/proposal_v1.xlsx
+++ b/docbuilder/data/templates/demo/proposal_v1.xlsx
@@ -89,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -99,6 +99,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -515,18 +518,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="4" t="n"/>
-      <c r="B1" s="4" t="n"/>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>[ LOGO ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="4" customHeight="1">
+      <c r="A2" s="3" t="n"/>
+      <c r="B2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="4" t="n"/>
+      <c r="B3" s="4" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
 </worksheet>

</xml_diff>